<commit_message>
Add six new 2025 entries without type/description
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KFNBQHEzPbML3vXDdVBdxh
</commit_message>
<xml_diff>
--- a/einnahmen/Einnahmen_Ausgaben_2025-2026.xlsx
+++ b/einnahmen/Einnahmen_Ausgaben_2025-2026.xlsx
@@ -712,20 +712,12 @@
     </row>
     <row r="7">
       <c r="A7" s="6" t="n">
-        <v>45716</v>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Ausgabe</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>Kontoführung</t>
-        </is>
-      </c>
+        <v>45688</v>
+      </c>
+      <c r="B7" s="7" t="n"/>
+      <c r="C7" s="8" t="n"/>
       <c r="D7" s="9" t="n">
-        <v>-15.9</v>
+        <v>385.5</v>
       </c>
       <c r="F7" s="10" t="n">
         <v>45717</v>
@@ -745,20 +737,12 @@
     </row>
     <row r="8">
       <c r="A8" s="6" t="n">
-        <v>45747</v>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Ausgabe</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>Kontoführung</t>
-        </is>
-      </c>
+        <v>45698</v>
+      </c>
+      <c r="B8" s="7" t="n"/>
+      <c r="C8" s="8" t="n"/>
       <c r="D8" s="9" t="n">
-        <v>-15.9</v>
+        <v>139.25</v>
       </c>
       <c r="F8" s="10" t="n">
         <v>45748</v>
@@ -778,20 +762,12 @@
     </row>
     <row r="9">
       <c r="A9" s="6" t="n">
-        <v>45748</v>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Einnahme</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>BP</t>
-        </is>
-      </c>
+        <v>45699</v>
+      </c>
+      <c r="B9" s="7" t="n"/>
+      <c r="C9" s="8" t="n"/>
       <c r="D9" s="9" t="n">
-        <v>385.5</v>
+        <v>-17.49</v>
       </c>
       <c r="F9" s="10" t="n">
         <v>45778</v>
@@ -811,20 +787,12 @@
     </row>
     <row r="10">
       <c r="A10" s="6" t="n">
-        <v>45748</v>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>Ausgabe</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>Domain</t>
-        </is>
-      </c>
+        <v>45699</v>
+      </c>
+      <c r="B10" s="7" t="n"/>
+      <c r="C10" s="8" t="n"/>
       <c r="D10" s="9" t="n">
-        <v>-7.95</v>
+        <v>-17.49</v>
       </c>
       <c r="F10" s="10" t="n">
         <v>45809</v>
@@ -844,20 +812,20 @@
     </row>
     <row r="11">
       <c r="A11" s="6" t="n">
-        <v>45757</v>
+        <v>45716</v>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Einnahme</t>
+          <t>Ausgabe</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>CC</t>
+          <t>Kontoführung</t>
         </is>
       </c>
       <c r="D11" s="9" t="n">
-        <v>500</v>
+        <v>-15.9</v>
       </c>
       <c r="F11" s="10" t="n">
         <v>45839</v>
@@ -877,20 +845,12 @@
     </row>
     <row r="12">
       <c r="A12" s="6" t="n">
-        <v>45763</v>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Ausgabe</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>MEB</t>
-        </is>
-      </c>
+        <v>45719</v>
+      </c>
+      <c r="B12" s="7" t="n"/>
+      <c r="C12" s="8" t="n"/>
       <c r="D12" s="9" t="n">
-        <v>-300</v>
+        <v>552.55</v>
       </c>
       <c r="F12" s="10" t="n">
         <v>45870</v>
@@ -910,20 +870,12 @@
     </row>
     <row r="13">
       <c r="A13" s="6" t="n">
-        <v>45777</v>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Ausgabe</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>MEB</t>
-        </is>
-      </c>
+        <v>45720</v>
+      </c>
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="8" t="n"/>
       <c r="D13" s="9" t="n">
-        <v>-300</v>
+        <v>-17.49</v>
       </c>
       <c r="F13" s="10" t="n">
         <v>45901</v>
@@ -943,7 +895,7 @@
     </row>
     <row r="14">
       <c r="A14" s="6" t="n">
-        <v>45777</v>
+        <v>45747</v>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
@@ -952,11 +904,11 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>MEB</t>
+          <t>Kontoführung</t>
         </is>
       </c>
       <c r="D14" s="9" t="n">
-        <v>-300</v>
+        <v>-15.9</v>
       </c>
       <c r="F14" s="10" t="n">
         <v>45931</v>
@@ -976,20 +928,20 @@
     </row>
     <row r="15">
       <c r="A15" s="6" t="n">
-        <v>45777</v>
+        <v>45748</v>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Ausgabe</t>
+          <t>Einnahme</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Kontoführung</t>
+          <t>BP</t>
         </is>
       </c>
       <c r="D15" s="9" t="n">
-        <v>-16.3</v>
+        <v>385.5</v>
       </c>
       <c r="F15" s="10" t="n">
         <v>45962</v>
@@ -1009,7 +961,7 @@
     </row>
     <row r="16">
       <c r="A16" s="6" t="n">
-        <v>45778</v>
+        <v>45748</v>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
@@ -1042,20 +994,20 @@
     </row>
     <row r="17">
       <c r="A17" s="6" t="n">
-        <v>45797</v>
+        <v>45757</v>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Ausgabe</t>
+          <t>Einnahme</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Domain</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="D17" s="9" t="n">
-        <v>-13.95</v>
+        <v>500</v>
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
@@ -1077,7 +1029,7 @@
     </row>
     <row r="18">
       <c r="A18" s="6" t="n">
-        <v>45804</v>
+        <v>45763</v>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
@@ -1090,25 +1042,25 @@
         </is>
       </c>
       <c r="D18" s="9" t="n">
-        <v>-150</v>
+        <v>-300</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n">
-        <v>45805</v>
+        <v>45777</v>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Einnahme</t>
+          <t>Ausgabe</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>CC</t>
+          <t>MEB</t>
         </is>
       </c>
       <c r="D19" s="9" t="n">
-        <v>1750</v>
+        <v>-300</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -1122,7 +1074,7 @@
     </row>
     <row r="20">
       <c r="A20" s="6" t="n">
-        <v>45807</v>
+        <v>45777</v>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
@@ -1135,17 +1087,17 @@
         </is>
       </c>
       <c r="D20" s="9" t="n">
-        <v>-750</v>
+        <v>-300</v>
       </c>
       <c r="F20" s="19" t="inlineStr">
         <is>
-          <t>(sollte 0 sein – sonst steht ein Datum aus einem anderen Jahr oder eine Zeile ohne Art in der Liste)</t>
+          <t>(sollte 0 sein – sonst fehlt bei einer Zeile die Art (Einnahme/Ausgabe) oder das Datum liegt in einem anderen Jahr)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="n">
-        <v>45807</v>
+        <v>45777</v>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
@@ -1158,12 +1110,12 @@
         </is>
       </c>
       <c r="D21" s="9" t="n">
-        <v>-17.1</v>
+        <v>-16.3</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="n">
-        <v>45807</v>
+        <v>45778</v>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
@@ -1172,34 +1124,34 @@
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>MEB</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="D22" s="9" t="n">
-        <v>-300</v>
+        <v>-7.95</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="n">
-        <v>45809</v>
+        <v>45797</v>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Einnahme</t>
+          <t>Ausgabe</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>BP</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="D23" s="9" t="n">
-        <v>359.8</v>
+        <v>-13.95</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="n">
-        <v>45811</v>
+        <v>45804</v>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
@@ -1208,34 +1160,34 @@
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>Domain</t>
+          <t>MEB</t>
         </is>
       </c>
       <c r="D24" s="9" t="n">
-        <v>-7.95</v>
+        <v>-150</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="n">
-        <v>45813</v>
+        <v>45805</v>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Ausgabe</t>
+          <t>Einnahme</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>Powercall</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="D25" s="9" t="n">
-        <v>-82.11</v>
+        <v>1750</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="n">
-        <v>45838</v>
+        <v>45807</v>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
@@ -1244,16 +1196,16 @@
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>Kontoführung</t>
+          <t>MEB</t>
         </is>
       </c>
       <c r="D26" s="9" t="n">
-        <v>-15.9</v>
+        <v>-750</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="n">
-        <v>45842</v>
+        <v>45807</v>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
@@ -1262,16 +1214,16 @@
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>Powercall</t>
+          <t>Kontoführung</t>
         </is>
       </c>
       <c r="D27" s="9" t="n">
-        <v>-82.11</v>
+        <v>-17.1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="n">
-        <v>45846</v>
+        <v>45807</v>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
@@ -1280,34 +1232,34 @@
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>Domain</t>
+          <t>MEB</t>
         </is>
       </c>
       <c r="D28" s="9" t="n">
-        <v>-7.95</v>
+        <v>-300</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="n">
-        <v>45854</v>
+        <v>45809</v>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Ausgabe</t>
+          <t>Einnahme</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>Jabra Headset</t>
+          <t>BP</t>
         </is>
       </c>
       <c r="D29" s="9" t="n">
-        <v>-152.81</v>
+        <v>359.8</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="n">
-        <v>45869</v>
+        <v>45811</v>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
@@ -1316,34 +1268,34 @@
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>Kontoführung</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="D30" s="9" t="n">
-        <v>-15.9</v>
+        <v>-7.95</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="n">
-        <v>45870</v>
+        <v>45813</v>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Einnahme</t>
+          <t>Ausgabe</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>CC</t>
+          <t>Powercall</t>
         </is>
       </c>
       <c r="D31" s="9" t="n">
-        <v>500</v>
+        <v>-82.11</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n">
-        <v>45873</v>
+        <v>45838</v>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
@@ -1352,16 +1304,16 @@
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>Domain</t>
+          <t>Kontoführung</t>
         </is>
       </c>
       <c r="D32" s="9" t="n">
-        <v>-7.95</v>
+        <v>-15.9</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="n">
-        <v>45874</v>
+        <v>45842</v>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
@@ -1379,25 +1331,25 @@
     </row>
     <row r="34">
       <c r="A34" s="6" t="n">
-        <v>45874</v>
+        <v>45846</v>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>Einnahme</t>
+          <t>Ausgabe</t>
         </is>
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="D34" s="9" t="n">
-        <v>100</v>
+        <v>-7.95</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="n">
-        <v>45898</v>
+        <v>45854</v>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
@@ -1406,16 +1358,16 @@
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Kontoführung</t>
+          <t>Jabra Headset</t>
         </is>
       </c>
       <c r="D35" s="9" t="n">
-        <v>-15.9</v>
+        <v>-152.81</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="n">
-        <v>45901</v>
+        <v>45869</v>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
@@ -1424,34 +1376,34 @@
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>Domain</t>
+          <t>Kontoführung</t>
         </is>
       </c>
       <c r="D36" s="9" t="n">
-        <v>-7.95</v>
+        <v>-15.9</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="n">
-        <v>45904</v>
+        <v>45870</v>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Ausgabe</t>
+          <t>Einnahme</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>Powercall</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="D37" s="9" t="n">
-        <v>-82.11</v>
+        <v>500</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n">
-        <v>45930</v>
+        <v>45873</v>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
@@ -1460,16 +1412,16 @@
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>Kontoführung</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="D38" s="9" t="n">
-        <v>-15.9</v>
+        <v>-7.95</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="n">
-        <v>45937</v>
+        <v>45874</v>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
@@ -1478,16 +1430,16 @@
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>Domain</t>
+          <t>Powercall</t>
         </is>
       </c>
       <c r="D39" s="9" t="n">
-        <v>-7.95</v>
+        <v>-82.11</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="n">
-        <v>45946</v>
+        <v>45874</v>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
@@ -1500,12 +1452,12 @@
         </is>
       </c>
       <c r="D40" s="9" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="n">
-        <v>45958</v>
+        <v>45898</v>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
@@ -1514,16 +1466,16 @@
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>Domain</t>
+          <t>Kontoführung</t>
         </is>
       </c>
       <c r="D41" s="9" t="n">
-        <v>-10.95</v>
+        <v>-15.9</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="n">
-        <v>45961</v>
+        <v>45901</v>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
@@ -1532,34 +1484,34 @@
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t>Kontoführung</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="D42" s="9" t="n">
-        <v>-16.1</v>
+        <v>-7.95</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="n">
-        <v>45962</v>
+        <v>45904</v>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Einnahme</t>
+          <t>Ausgabe</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>Powercall</t>
         </is>
       </c>
       <c r="D43" s="9" t="n">
-        <v>134.46</v>
+        <v>-82.11</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="n">
-        <v>45989</v>
+        <v>45930</v>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
@@ -1568,16 +1520,16 @@
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>Domain</t>
+          <t>Kontoführung</t>
         </is>
       </c>
       <c r="D44" s="9" t="n">
-        <v>-7.5</v>
+        <v>-15.9</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="n">
-        <v>45989</v>
+        <v>45937</v>
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
@@ -1586,16 +1538,16 @@
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>Kontoführung</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="D45" s="9" t="n">
-        <v>-15.9</v>
+        <v>-7.95</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="n">
-        <v>45992</v>
+        <v>45946</v>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
@@ -1604,66 +1556,138 @@
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D46" s="9" t="n">
-        <v>564.64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="n">
+        <v>45958</v>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Ausgabe</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="n">
+        <v>-10.95</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="n">
+        <v>45961</v>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Ausgabe</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>Kontoführung</t>
+        </is>
+      </c>
+      <c r="D48" s="9" t="n">
+        <v>-16.1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="n">
+        <v>45962</v>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Einnahme</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="D49" s="9" t="n">
+        <v>134.46</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="n">
+        <v>45989</v>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Ausgabe</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="D50" s="9" t="n">
+        <v>-7.5</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="n">
+        <v>45989</v>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Ausgabe</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>Kontoführung</t>
+        </is>
+      </c>
+      <c r="D51" s="9" t="n">
+        <v>-15.9</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="n">
+        <v>45992</v>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Einnahme</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="D52" s="9" t="n">
+        <v>564.64</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="n">
         <v>46022</v>
       </c>
-      <c r="B47" s="7" t="inlineStr">
+      <c r="B53" s="7" t="inlineStr">
         <is>
           <t>Ausgabe</t>
         </is>
       </c>
-      <c r="C47" s="8" t="inlineStr">
+      <c r="C53" s="8" t="inlineStr">
         <is>
           <t>Kontoführung</t>
         </is>
       </c>
-      <c r="D47" s="9" t="n">
+      <c r="D53" s="9" t="n">
         <v>-15.9</v>
       </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="6" t="n"/>
-      <c r="B48" s="7" t="n"/>
-      <c r="C48" s="8" t="n"/>
-      <c r="D48" s="9" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="6" t="n"/>
-      <c r="B49" s="7" t="n"/>
-      <c r="C49" s="8" t="n"/>
-      <c r="D49" s="9" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="6" t="n"/>
-      <c r="B50" s="7" t="n"/>
-      <c r="C50" s="8" t="n"/>
-      <c r="D50" s="9" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="6" t="n"/>
-      <c r="B51" s="7" t="n"/>
-      <c r="C51" s="8" t="n"/>
-      <c r="D51" s="9" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="6" t="n"/>
-      <c r="B52" s="7" t="n"/>
-      <c r="C52" s="8" t="n"/>
-      <c r="D52" s="9" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="6" t="n"/>
-      <c r="B53" s="7" t="n"/>
-      <c r="C53" s="8" t="n"/>
-      <c r="D53" s="9" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="6" t="n"/>
@@ -3772,7 +3796,7 @@
       </c>
       <c r="F20" s="19" t="inlineStr">
         <is>
-          <t>(sollte 0 sein – sonst steht ein Datum aus einem anderen Jahr oder eine Zeile ohne Art in der Liste)</t>
+          <t>(sollte 0 sein – sonst fehlt bei einer Zeile die Art (Einnahme/Ausgabe) oder das Datum liegt in einem anderen Jahr)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add further 2025 and 2026 entries without type/description
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KFNBQHEzPbML3vXDdVBdxh
</commit_message>
<xml_diff>
--- a/einnahmen/Einnahmen_Ausgaben_2025-2026.xlsx
+++ b/einnahmen/Einnahmen_Ausgaben_2025-2026.xlsx
@@ -870,12 +870,12 @@
     </row>
     <row r="13">
       <c r="A13" s="6" t="n">
-        <v>45720</v>
+        <v>45719</v>
       </c>
       <c r="B13" s="7" t="n"/>
       <c r="C13" s="8" t="n"/>
       <c r="D13" s="9" t="n">
-        <v>-17.49</v>
+        <v>42.26</v>
       </c>
       <c r="F13" s="10" t="n">
         <v>45901</v>
@@ -895,20 +895,12 @@
     </row>
     <row r="14">
       <c r="A14" s="6" t="n">
-        <v>45747</v>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Ausgabe</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Kontoführung</t>
-        </is>
-      </c>
+        <v>45720</v>
+      </c>
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="8" t="n"/>
       <c r="D14" s="9" t="n">
-        <v>-15.9</v>
+        <v>-17.49</v>
       </c>
       <c r="F14" s="10" t="n">
         <v>45931</v>
@@ -928,20 +920,20 @@
     </row>
     <row r="15">
       <c r="A15" s="6" t="n">
-        <v>45748</v>
+        <v>45747</v>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Einnahme</t>
+          <t>Ausgabe</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>BP</t>
+          <t>Kontoführung</t>
         </is>
       </c>
       <c r="D15" s="9" t="n">
-        <v>385.5</v>
+        <v>-15.9</v>
       </c>
       <c r="F15" s="10" t="n">
         <v>45962</v>
@@ -965,16 +957,16 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Ausgabe</t>
+          <t>Einnahme</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Domain</t>
+          <t>BP</t>
         </is>
       </c>
       <c r="D16" s="9" t="n">
-        <v>-7.95</v>
+        <v>385.5</v>
       </c>
       <c r="F16" s="10" t="n">
         <v>45992</v>
@@ -994,20 +986,20 @@
     </row>
     <row r="17">
       <c r="A17" s="6" t="n">
-        <v>45757</v>
+        <v>45748</v>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Einnahme</t>
+          <t>Ausgabe</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>CC</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="D17" s="9" t="n">
-        <v>500</v>
+        <v>-7.95</v>
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
@@ -1029,25 +1021,25 @@
     </row>
     <row r="18">
       <c r="A18" s="6" t="n">
-        <v>45763</v>
+        <v>45757</v>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Ausgabe</t>
+          <t>Einnahme</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>MEB</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="D18" s="9" t="n">
-        <v>-300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n">
-        <v>45777</v>
+        <v>45763</v>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
@@ -1106,16 +1098,16 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>Kontoführung</t>
+          <t>MEB</t>
         </is>
       </c>
       <c r="D21" s="9" t="n">
-        <v>-16.3</v>
+        <v>-300</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="n">
-        <v>45778</v>
+        <v>45777</v>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
@@ -1124,16 +1116,16 @@
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>Domain</t>
+          <t>Kontoführung</t>
         </is>
       </c>
       <c r="D22" s="9" t="n">
-        <v>-7.95</v>
+        <v>-16.3</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="n">
-        <v>45797</v>
+        <v>45778</v>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
@@ -1146,12 +1138,12 @@
         </is>
       </c>
       <c r="D23" s="9" t="n">
-        <v>-13.95</v>
+        <v>-7.95</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="n">
-        <v>45804</v>
+        <v>45797</v>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
@@ -1160,47 +1152,47 @@
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>MEB</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="D24" s="9" t="n">
-        <v>-150</v>
+        <v>-13.95</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="n">
-        <v>45805</v>
+        <v>45804</v>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Einnahme</t>
+          <t>Ausgabe</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>CC</t>
+          <t>MEB</t>
         </is>
       </c>
       <c r="D25" s="9" t="n">
-        <v>1750</v>
+        <v>-150</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="n">
-        <v>45807</v>
+        <v>45805</v>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Ausgabe</t>
+          <t>Einnahme</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>MEB</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="D26" s="9" t="n">
-        <v>-750</v>
+        <v>1750</v>
       </c>
     </row>
     <row r="27">
@@ -1214,11 +1206,11 @@
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>Kontoführung</t>
+          <t>MEB</t>
         </is>
       </c>
       <c r="D27" s="9" t="n">
-        <v>-17.1</v>
+        <v>-750</v>
       </c>
     </row>
     <row r="28">
@@ -1232,52 +1224,52 @@
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>MEB</t>
+          <t>Kontoführung</t>
         </is>
       </c>
       <c r="D28" s="9" t="n">
-        <v>-300</v>
+        <v>-17.1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="n">
-        <v>45809</v>
+        <v>45807</v>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Einnahme</t>
+          <t>Ausgabe</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>BP</t>
+          <t>MEB</t>
         </is>
       </c>
       <c r="D29" s="9" t="n">
-        <v>359.8</v>
+        <v>-300</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="n">
-        <v>45811</v>
+        <v>45809</v>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Ausgabe</t>
+          <t>Einnahme</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>Domain</t>
+          <t>BP</t>
         </is>
       </c>
       <c r="D30" s="9" t="n">
-        <v>-7.95</v>
+        <v>359.8</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="n">
-        <v>45813</v>
+        <v>45811</v>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
@@ -1286,16 +1278,16 @@
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>Powercall</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="D31" s="9" t="n">
-        <v>-82.11</v>
+        <v>-7.95</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n">
-        <v>45838</v>
+        <v>45813</v>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
@@ -1304,16 +1296,16 @@
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>Kontoführung</t>
+          <t>Powercall</t>
         </is>
       </c>
       <c r="D32" s="9" t="n">
-        <v>-15.9</v>
+        <v>-82.11</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="n">
-        <v>45842</v>
+        <v>45838</v>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
@@ -1322,16 +1314,16 @@
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>Powercall</t>
+          <t>Kontoführung</t>
         </is>
       </c>
       <c r="D33" s="9" t="n">
-        <v>-82.11</v>
+        <v>-15.9</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="n">
-        <v>45846</v>
+        <v>45842</v>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
@@ -1340,16 +1332,16 @@
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>Domain</t>
+          <t>Powercall</t>
         </is>
       </c>
       <c r="D34" s="9" t="n">
-        <v>-7.95</v>
+        <v>-82.11</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="n">
-        <v>45854</v>
+        <v>45846</v>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
@@ -1358,16 +1350,16 @@
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Jabra Headset</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="D35" s="9" t="n">
-        <v>-152.81</v>
+        <v>-7.95</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="n">
-        <v>45869</v>
+        <v>45854</v>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
@@ -1376,52 +1368,52 @@
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>Kontoführung</t>
+          <t>Jabra Headset</t>
         </is>
       </c>
       <c r="D36" s="9" t="n">
-        <v>-15.9</v>
+        <v>-152.81</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="n">
-        <v>45870</v>
+        <v>45869</v>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Einnahme</t>
+          <t>Ausgabe</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>CC</t>
+          <t>Kontoführung</t>
         </is>
       </c>
       <c r="D37" s="9" t="n">
-        <v>500</v>
+        <v>-15.9</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n">
-        <v>45873</v>
+        <v>45870</v>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>Ausgabe</t>
+          <t>Einnahme</t>
         </is>
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>Domain</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="D38" s="9" t="n">
-        <v>-7.95</v>
+        <v>500</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="n">
-        <v>45874</v>
+        <v>45873</v>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
@@ -1430,11 +1422,11 @@
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>Powercall</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="D39" s="9" t="n">
-        <v>-82.11</v>
+        <v>-7.95</v>
       </c>
     </row>
     <row r="40">
@@ -1443,39 +1435,39 @@
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>Einnahme</t>
+          <t>Ausgabe</t>
         </is>
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Powercall</t>
         </is>
       </c>
       <c r="D40" s="9" t="n">
-        <v>100</v>
+        <v>-82.11</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="n">
-        <v>45898</v>
+        <v>45874</v>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Ausgabe</t>
+          <t>Einnahme</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>Kontoführung</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D41" s="9" t="n">
-        <v>-15.9</v>
+        <v>100</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="n">
-        <v>45901</v>
+        <v>45898</v>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
@@ -1484,16 +1476,16 @@
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t>Domain</t>
+          <t>Kontoführung</t>
         </is>
       </c>
       <c r="D42" s="9" t="n">
-        <v>-7.95</v>
+        <v>-15.9</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="n">
-        <v>45904</v>
+        <v>45901</v>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
@@ -1502,16 +1494,16 @@
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>Powercall</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="D43" s="9" t="n">
-        <v>-82.11</v>
+        <v>-7.95</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="n">
-        <v>45930</v>
+        <v>45904</v>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
@@ -1520,16 +1512,16 @@
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>Kontoführung</t>
+          <t>Powercall</t>
         </is>
       </c>
       <c r="D44" s="9" t="n">
-        <v>-15.9</v>
+        <v>-82.11</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="n">
-        <v>45937</v>
+        <v>45930</v>
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
@@ -1538,52 +1530,52 @@
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>Domain</t>
+          <t>Kontoführung</t>
         </is>
       </c>
       <c r="D45" s="9" t="n">
-        <v>-7.95</v>
+        <v>-15.9</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="n">
-        <v>45946</v>
+        <v>45937</v>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>Einnahme</t>
+          <t>Ausgabe</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="D46" s="9" t="n">
-        <v>60</v>
+        <v>-7.95</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="n">
-        <v>45958</v>
+        <v>45946</v>
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>Ausgabe</t>
+          <t>Einnahme</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>Domain</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D47" s="9" t="n">
-        <v>-10.95</v>
+        <v>60</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="n">
-        <v>45961</v>
+        <v>45958</v>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
@@ -1592,47 +1584,47 @@
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>Kontoführung</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="D48" s="9" t="n">
-        <v>-16.1</v>
+        <v>-10.95</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="n">
-        <v>45962</v>
+        <v>45961</v>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Einnahme</t>
+          <t>Ausgabe</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>Kontoführung</t>
         </is>
       </c>
       <c r="D49" s="9" t="n">
-        <v>134.46</v>
+        <v>-16.1</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="n">
-        <v>45989</v>
+        <v>45962</v>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>Ausgabe</t>
+          <t>Einnahme</t>
         </is>
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>Domain</t>
+          <t>SF</t>
         </is>
       </c>
       <c r="D50" s="9" t="n">
-        <v>-7.5</v>
+        <v>134.46</v>
       </c>
     </row>
     <row r="51">
@@ -1646,54 +1638,66 @@
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>Kontoführung</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="D51" s="9" t="n">
-        <v>-15.9</v>
+        <v>-7.5</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="6" t="n">
-        <v>45992</v>
+        <v>45989</v>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>Einnahme</t>
+          <t>Ausgabe</t>
         </is>
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>Kontoführung</t>
         </is>
       </c>
       <c r="D52" s="9" t="n">
-        <v>564.64</v>
+        <v>-15.9</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="6" t="n">
+        <v>45992</v>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Einnahme</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="D53" s="9" t="n">
+        <v>564.64</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="n">
         <v>46022</v>
       </c>
-      <c r="B53" s="7" t="inlineStr">
+      <c r="B54" s="7" t="inlineStr">
         <is>
           <t>Ausgabe</t>
         </is>
       </c>
-      <c r="C53" s="8" t="inlineStr">
+      <c r="C54" s="8" t="inlineStr">
         <is>
           <t>Kontoführung</t>
         </is>
       </c>
-      <c r="D53" s="9" t="n">
+      <c r="D54" s="9" t="n">
         <v>-15.9</v>
       </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="6" t="n"/>
-      <c r="B54" s="7" t="n"/>
-      <c r="C54" s="8" t="n"/>
-      <c r="D54" s="9" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="6" t="n"/>
@@ -3336,20 +3340,12 @@
     </row>
     <row r="6">
       <c r="A6" s="6" t="n">
-        <v>46063</v>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Einnahme</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
+        <v>46052</v>
+      </c>
+      <c r="B6" s="7" t="n"/>
+      <c r="C6" s="8" t="n"/>
       <c r="D6" s="9" t="n">
-        <v>405.73</v>
+        <v>-15.9</v>
       </c>
       <c r="F6" s="10" t="n">
         <v>46054</v>
@@ -3369,7 +3365,7 @@
     </row>
     <row r="7">
       <c r="A7" s="6" t="n">
-        <v>46091</v>
+        <v>46063</v>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
@@ -3382,7 +3378,7 @@
         </is>
       </c>
       <c r="D7" s="9" t="n">
-        <v>544.42</v>
+        <v>405.73</v>
       </c>
       <c r="F7" s="10" t="n">
         <v>46082</v>
@@ -3402,20 +3398,12 @@
     </row>
     <row r="8">
       <c r="A8" s="6" t="n">
-        <v>46122</v>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Einnahme</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
+        <v>46080</v>
+      </c>
+      <c r="B8" s="7" t="n"/>
+      <c r="C8" s="8" t="n"/>
       <c r="D8" s="9" t="n">
-        <v>446.89</v>
+        <v>-15.9</v>
       </c>
       <c r="F8" s="10" t="n">
         <v>46113</v>
@@ -3435,20 +3423,20 @@
     </row>
     <row r="9">
       <c r="A9" s="6" t="n">
-        <v>46132</v>
+        <v>46091</v>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Ausgabe</t>
+          <t>Einnahme</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="D9" s="9" t="n">
-        <v>-21.42</v>
+        <v>544.42</v>
       </c>
       <c r="F9" s="10" t="n">
         <v>46143</v>
@@ -3468,20 +3456,12 @@
     </row>
     <row r="10">
       <c r="A10" s="6" t="n">
-        <v>46150</v>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>Einnahme</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
+        <v>46092</v>
+      </c>
+      <c r="B10" s="7" t="n"/>
+      <c r="C10" s="8" t="n"/>
       <c r="D10" s="9" t="n">
-        <v>575.52</v>
+        <v>-32.25</v>
       </c>
       <c r="F10" s="10" t="n">
         <v>46174</v>
@@ -3501,20 +3481,12 @@
     </row>
     <row r="11">
       <c r="A11" s="6" t="n">
-        <v>46183</v>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Einnahme</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
+        <v>46112</v>
+      </c>
+      <c r="B11" s="7" t="n"/>
+      <c r="C11" s="8" t="n"/>
       <c r="D11" s="9" t="n">
-        <v>560.23</v>
+        <v>-15.9</v>
       </c>
       <c r="F11" s="10" t="n">
         <v>46204</v>
@@ -3534,20 +3506,20 @@
     </row>
     <row r="12">
       <c r="A12" s="6" t="n">
-        <v>46191</v>
+        <v>46122</v>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Ausgabe</t>
+          <t>Einnahme</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>V2T</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="D12" s="9" t="n">
-        <v>-39.9</v>
+        <v>446.89</v>
       </c>
       <c r="F12" s="10" t="n">
         <v>46235</v>
@@ -3567,7 +3539,7 @@
     </row>
     <row r="13">
       <c r="A13" s="6" t="n">
-        <v>46202</v>
+        <v>46132</v>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
@@ -3576,11 +3548,11 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Domain</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="D13" s="9" t="n">
-        <v>-7.95</v>
+        <v>-21.42</v>
       </c>
       <c r="F13" s="10" t="n">
         <v>46266</v>
@@ -3600,20 +3572,12 @@
     </row>
     <row r="14">
       <c r="A14" s="6" t="n">
-        <v>46213</v>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Einnahme</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
+        <v>46142</v>
+      </c>
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="8" t="n"/>
       <c r="D14" s="9" t="n">
-        <v>178.48</v>
+        <v>-15.9</v>
       </c>
       <c r="F14" s="10" t="n">
         <v>46296</v>
@@ -3633,20 +3597,20 @@
     </row>
     <row r="15">
       <c r="A15" s="6" t="n">
-        <v>46223</v>
+        <v>46150</v>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Ausgabe</t>
+          <t>Einnahme</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="D15" s="9" t="n">
-        <v>-21.42</v>
+        <v>575.52</v>
       </c>
       <c r="F15" s="10" t="n">
         <v>46327</v>
@@ -3666,20 +3630,12 @@
     </row>
     <row r="16">
       <c r="A16" s="6" t="n">
-        <v>46232</v>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>Ausgabe</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>Whoop</t>
-        </is>
-      </c>
+        <v>46154</v>
+      </c>
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="8" t="n"/>
       <c r="D16" s="9" t="n">
-        <v>-11.89</v>
+        <v>-15.9</v>
       </c>
       <c r="F16" s="10" t="n">
         <v>46357</v>
@@ -3699,20 +3655,12 @@
     </row>
     <row r="17">
       <c r="A17" s="6" t="n">
-        <v>46244</v>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>Einnahme</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
+        <v>46161</v>
+      </c>
+      <c r="B17" s="7" t="n"/>
+      <c r="C17" s="8" t="n"/>
       <c r="D17" s="9" t="n">
-        <v>420.07</v>
+        <v>-21.42</v>
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
@@ -3734,38 +3682,30 @@
     </row>
     <row r="18">
       <c r="A18" s="6" t="n">
-        <v>46252</v>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>Ausgabe</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>Claude</t>
-        </is>
-      </c>
+        <v>46171</v>
+      </c>
+      <c r="B18" s="7" t="n"/>
+      <c r="C18" s="8" t="n"/>
       <c r="D18" s="9" t="n">
-        <v>-21.42</v>
+        <v>-15.9</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n">
-        <v>46262</v>
+        <v>46183</v>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Ausgabe</t>
+          <t>Einnahme</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Whoop</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="D19" s="9" t="n">
-        <v>-11.89</v>
+        <v>560.23</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -3779,20 +3719,20 @@
     </row>
     <row r="20">
       <c r="A20" s="6" t="n">
-        <v>46275</v>
+        <v>46191</v>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Einnahme</t>
+          <t>Ausgabe</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>V2T</t>
         </is>
       </c>
       <c r="D20" s="9" t="n">
-        <v>344.78</v>
+        <v>-39.9</v>
       </c>
       <c r="F20" s="19" t="inlineStr">
         <is>
@@ -3802,7 +3742,7 @@
     </row>
     <row r="21">
       <c r="A21" s="6" t="n">
-        <v>46283</v>
+        <v>46202</v>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
@@ -3811,34 +3751,26 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="D21" s="9" t="n">
-        <v>-21.42</v>
+        <v>-7.95</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="n">
-        <v>46294</v>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>Ausgabe</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>Whoop</t>
-        </is>
-      </c>
+        <v>46203</v>
+      </c>
+      <c r="B22" s="7" t="n"/>
+      <c r="C22" s="8" t="n"/>
       <c r="D22" s="9" t="n">
-        <v>-11.89</v>
+        <v>-15.9</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="n">
-        <v>46304</v>
+        <v>46213</v>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
@@ -3851,80 +3783,200 @@
         </is>
       </c>
       <c r="D23" s="9" t="n">
-        <v>215.33</v>
+        <v>178.48</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="n"/>
-      <c r="B24" s="7" t="n"/>
-      <c r="C24" s="8" t="n"/>
-      <c r="D24" s="9" t="n"/>
+      <c r="A24" s="6" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Ausgabe</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="n">
+        <v>-21.42</v>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="n"/>
-      <c r="B25" s="7" t="n"/>
-      <c r="C25" s="8" t="n"/>
-      <c r="D25" s="9" t="n"/>
+      <c r="A25" s="6" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Ausgabe</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Whoop</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="n">
+        <v>-11.89</v>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="n"/>
+      <c r="A26" s="6" t="n">
+        <v>46234</v>
+      </c>
       <c r="B26" s="7" t="n"/>
       <c r="C26" s="8" t="n"/>
-      <c r="D26" s="9" t="n"/>
+      <c r="D26" s="9" t="n">
+        <v>-15.9</v>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="n"/>
-      <c r="B27" s="7" t="n"/>
-      <c r="C27" s="8" t="n"/>
-      <c r="D27" s="9" t="n"/>
+      <c r="A27" s="6" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Einnahme</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="n">
+        <v>420.07</v>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="n"/>
-      <c r="B28" s="7" t="n"/>
-      <c r="C28" s="8" t="n"/>
-      <c r="D28" s="9" t="n"/>
+      <c r="A28" s="6" t="n">
+        <v>46252</v>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Ausgabe</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="n">
+        <v>-21.42</v>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="n"/>
-      <c r="B29" s="7" t="n"/>
-      <c r="C29" s="8" t="n"/>
-      <c r="D29" s="9" t="n"/>
+      <c r="A29" s="6" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Ausgabe</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Whoop</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="n">
+        <v>-11.89</v>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="n"/>
+      <c r="A30" s="6" t="n">
+        <v>46265</v>
+      </c>
       <c r="B30" s="7" t="n"/>
       <c r="C30" s="8" t="n"/>
-      <c r="D30" s="9" t="n"/>
+      <c r="D30" s="9" t="n">
+        <v>-15.9</v>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="n"/>
-      <c r="B31" s="7" t="n"/>
-      <c r="C31" s="8" t="n"/>
-      <c r="D31" s="9" t="n"/>
+      <c r="A31" s="6" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Einnahme</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="n">
+        <v>344.78</v>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="n"/>
-      <c r="B32" s="7" t="n"/>
-      <c r="C32" s="8" t="n"/>
-      <c r="D32" s="9" t="n"/>
+      <c r="A32" s="6" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Ausgabe</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="n">
+        <v>-21.42</v>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="n"/>
-      <c r="B33" s="7" t="n"/>
-      <c r="C33" s="8" t="n"/>
-      <c r="D33" s="9" t="n"/>
+      <c r="A33" s="6" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Ausgabe</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Whoop</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="n">
+        <v>-11.89</v>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="n"/>
+      <c r="A34" s="6" t="n">
+        <v>46295</v>
+      </c>
       <c r="B34" s="7" t="n"/>
       <c r="C34" s="8" t="n"/>
-      <c r="D34" s="9" t="n"/>
+      <c r="D34" s="9" t="n">
+        <v>-15.9</v>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="n"/>
-      <c r="B35" s="7" t="n"/>
-      <c r="C35" s="8" t="n"/>
-      <c r="D35" s="9" t="n"/>
+      <c r="A35" s="6" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Einnahme</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="n">
+        <v>215.33</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="n"/>

</xml_diff>

<commit_message>
Übersicht: show 2025 table from April only
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KFNBQHEzPbML3vXDdVBdxh
</commit_message>
<xml_diff>
--- a/einnahmen/Einnahmen_Ausgaben_2025-2026.xlsx
+++ b/einnahmen/Einnahmen_Ausgaben_2025-2026.xlsx
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:D33"/>
+  <dimension ref="A2:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="23" min="1" max="1"/>
@@ -536,6 +536,7 @@
     <col width="16" customWidth="1" style="23" min="4" max="4"/>
   </cols>
   <sheetData>
+    <row r="1" s="23"/>
     <row r="2" ht="30" customHeight="1" s="23">
       <c r="A2" s="24" t="inlineStr">
         <is>
@@ -558,500 +559,459 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" s="23">
       <c r="A3" s="10">
-        <f>'2025'!F5</f>
+        <f>'2025'!F8</f>
         <v/>
       </c>
       <c r="B3" s="11">
-        <f>'2025'!G5</f>
+        <f>'2025'!G8</f>
         <v/>
       </c>
       <c r="C3" s="12">
-        <f>'2025'!H5</f>
+        <f>'2025'!H8</f>
         <v/>
       </c>
       <c r="D3" s="13">
-        <f>'2025'!I5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4">
+        <f>'2025'!I8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4" s="23">
       <c r="A4" s="10">
-        <f>'2025'!F6</f>
+        <f>'2025'!F9</f>
         <v/>
       </c>
       <c r="B4" s="11">
-        <f>'2025'!G6</f>
+        <f>'2025'!G9</f>
         <v/>
       </c>
       <c r="C4" s="12">
-        <f>'2025'!H6</f>
+        <f>'2025'!H9</f>
         <v/>
       </c>
       <c r="D4" s="13">
-        <f>'2025'!I6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
+        <f>'2025'!I9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" s="23">
       <c r="A5" s="10">
-        <f>'2025'!F7</f>
+        <f>'2025'!F10</f>
         <v/>
       </c>
       <c r="B5" s="11">
-        <f>'2025'!G7</f>
+        <f>'2025'!G10</f>
         <v/>
       </c>
       <c r="C5" s="12">
-        <f>'2025'!H7</f>
+        <f>'2025'!H10</f>
         <v/>
       </c>
       <c r="D5" s="13">
-        <f>'2025'!I7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
+        <f>'2025'!I10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" s="23">
       <c r="A6" s="10">
-        <f>'2025'!F8</f>
+        <f>'2025'!F11</f>
         <v/>
       </c>
       <c r="B6" s="11">
-        <f>'2025'!G8</f>
+        <f>'2025'!G11</f>
         <v/>
       </c>
       <c r="C6" s="12">
-        <f>'2025'!H8</f>
+        <f>'2025'!H11</f>
         <v/>
       </c>
       <c r="D6" s="13">
-        <f>'2025'!I8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
+        <f>'2025'!I11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" s="23">
       <c r="A7" s="10">
-        <f>'2025'!F9</f>
+        <f>'2025'!F12</f>
         <v/>
       </c>
       <c r="B7" s="11">
-        <f>'2025'!G9</f>
+        <f>'2025'!G12</f>
         <v/>
       </c>
       <c r="C7" s="12">
-        <f>'2025'!H9</f>
+        <f>'2025'!H12</f>
         <v/>
       </c>
       <c r="D7" s="13">
-        <f>'2025'!I9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
+        <f>'2025'!I12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" s="23">
       <c r="A8" s="10">
-        <f>'2025'!F10</f>
+        <f>'2025'!F13</f>
         <v/>
       </c>
       <c r="B8" s="11">
-        <f>'2025'!G10</f>
+        <f>'2025'!G13</f>
         <v/>
       </c>
       <c r="C8" s="12">
-        <f>'2025'!H10</f>
+        <f>'2025'!H13</f>
         <v/>
       </c>
       <c r="D8" s="13">
-        <f>'2025'!I10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
+        <f>'2025'!I13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" s="23">
       <c r="A9" s="10">
-        <f>'2025'!F11</f>
+        <f>'2025'!F14</f>
         <v/>
       </c>
       <c r="B9" s="11">
-        <f>'2025'!G11</f>
+        <f>'2025'!G14</f>
         <v/>
       </c>
       <c r="C9" s="12">
-        <f>'2025'!H11</f>
+        <f>'2025'!H14</f>
         <v/>
       </c>
       <c r="D9" s="13">
-        <f>'2025'!I11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
+        <f>'2025'!I14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" s="23">
       <c r="A10" s="10">
-        <f>'2025'!F12</f>
+        <f>'2025'!F15</f>
         <v/>
       </c>
       <c r="B10" s="11">
-        <f>'2025'!G12</f>
+        <f>'2025'!G15</f>
         <v/>
       </c>
       <c r="C10" s="12">
-        <f>'2025'!H12</f>
+        <f>'2025'!H15</f>
         <v/>
       </c>
       <c r="D10" s="13">
-        <f>'2025'!I12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
+        <f>'2025'!I15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" s="23">
       <c r="A11" s="10">
-        <f>'2025'!F13</f>
+        <f>'2025'!F16</f>
         <v/>
       </c>
       <c r="B11" s="11">
-        <f>'2025'!G13</f>
+        <f>'2025'!G16</f>
         <v/>
       </c>
       <c r="C11" s="12">
-        <f>'2025'!H13</f>
+        <f>'2025'!H16</f>
         <v/>
       </c>
       <c r="D11" s="13">
-        <f>'2025'!I13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="10">
-        <f>'2025'!F14</f>
-        <v/>
-      </c>
-      <c r="B12" s="11">
-        <f>'2025'!G14</f>
-        <v/>
-      </c>
-      <c r="C12" s="12">
-        <f>'2025'!H14</f>
-        <v/>
-      </c>
-      <c r="D12" s="13">
-        <f>'2025'!I14</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="10">
-        <f>'2025'!F15</f>
-        <v/>
-      </c>
-      <c r="B13" s="11">
-        <f>'2025'!G15</f>
-        <v/>
-      </c>
-      <c r="C13" s="12">
-        <f>'2025'!H15</f>
-        <v/>
-      </c>
-      <c r="D13" s="13">
-        <f>'2025'!I15</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="10">
-        <f>'2025'!F16</f>
-        <v/>
-      </c>
-      <c r="B14" s="11">
-        <f>'2025'!G16</f>
-        <v/>
-      </c>
-      <c r="C14" s="12">
-        <f>'2025'!H16</f>
-        <v/>
-      </c>
-      <c r="D14" s="13">
         <f>'2025'!I16</f>
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="16" t="inlineStr">
-        <is>
-          <t>Gesamt 2025</t>
-        </is>
-      </c>
-      <c r="B15" s="17">
-        <f>'2025'!G17</f>
-        <v/>
-      </c>
-      <c r="C15" s="18">
-        <f>'2025'!H17</f>
-        <v/>
-      </c>
-      <c r="D15" s="19">
-        <f>'2025'!I17</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1" s="23">
-      <c r="A20" s="24" t="inlineStr">
+    <row r="12" s="23">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>Gesamt 2025 (ab April)</t>
+        </is>
+      </c>
+      <c r="B12" s="17">
+        <f>SUM(B3:B11)</f>
+        <v/>
+      </c>
+      <c r="C12" s="18">
+        <f>SUM(C3:C11)</f>
+        <v/>
+      </c>
+      <c r="D12" s="19">
+        <f>SUM(D3:D11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" s="23"/>
+    <row r="14" s="23"/>
+    <row r="15" s="23"/>
+    <row r="16" s="23"/>
+    <row r="17" ht="30" customHeight="1" s="23">
+      <c r="A17" s="24" t="inlineStr">
         <is>
           <t>Monat 2026</t>
         </is>
       </c>
-      <c r="B20" s="25" t="inlineStr">
+      <c r="B17" s="25" t="inlineStr">
         <is>
           <t>Einnahmen (€)</t>
         </is>
       </c>
-      <c r="C20" s="26" t="inlineStr">
+      <c r="C17" s="26" t="inlineStr">
         <is>
           <t>Ausgaben (€)</t>
         </is>
       </c>
-      <c r="D20" s="24" t="inlineStr">
+      <c r="D17" s="24" t="inlineStr">
         <is>
           <t>Differenz (€)</t>
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="18" s="23">
+      <c r="A18" s="10">
+        <f>'2026'!F5</f>
+        <v/>
+      </c>
+      <c r="B18" s="11">
+        <f>'2026'!G5</f>
+        <v/>
+      </c>
+      <c r="C18" s="12">
+        <f>'2026'!H5</f>
+        <v/>
+      </c>
+      <c r="D18" s="13">
+        <f>'2026'!I5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" s="23">
+      <c r="A19" s="10">
+        <f>'2026'!F6</f>
+        <v/>
+      </c>
+      <c r="B19" s="11">
+        <f>'2026'!G6</f>
+        <v/>
+      </c>
+      <c r="C19" s="12">
+        <f>'2026'!H6</f>
+        <v/>
+      </c>
+      <c r="D19" s="13">
+        <f>'2026'!I6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" s="23">
+      <c r="A20" s="10">
+        <f>'2026'!F7</f>
+        <v/>
+      </c>
+      <c r="B20" s="11">
+        <f>'2026'!G7</f>
+        <v/>
+      </c>
+      <c r="C20" s="12">
+        <f>'2026'!H7</f>
+        <v/>
+      </c>
+      <c r="D20" s="13">
+        <f>'2026'!I7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" s="23">
       <c r="A21" s="10">
-        <f>'2026'!F5</f>
+        <f>'2026'!F8</f>
         <v/>
       </c>
       <c r="B21" s="11">
-        <f>'2026'!G5</f>
+        <f>'2026'!G8</f>
         <v/>
       </c>
       <c r="C21" s="12">
-        <f>'2026'!H5</f>
+        <f>'2026'!H8</f>
         <v/>
       </c>
       <c r="D21" s="13">
-        <f>'2026'!I5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
+        <f>'2026'!I8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" s="23">
       <c r="A22" s="10">
-        <f>'2026'!F6</f>
+        <f>'2026'!F9</f>
         <v/>
       </c>
       <c r="B22" s="11">
-        <f>'2026'!G6</f>
+        <f>'2026'!G9</f>
         <v/>
       </c>
       <c r="C22" s="12">
-        <f>'2026'!H6</f>
+        <f>'2026'!H9</f>
         <v/>
       </c>
       <c r="D22" s="13">
-        <f>'2026'!I6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
+        <f>'2026'!I9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" s="23">
       <c r="A23" s="10">
-        <f>'2026'!F7</f>
+        <f>'2026'!F10</f>
         <v/>
       </c>
       <c r="B23" s="11">
-        <f>'2026'!G7</f>
+        <f>'2026'!G10</f>
         <v/>
       </c>
       <c r="C23" s="12">
-        <f>'2026'!H7</f>
+        <f>'2026'!H10</f>
         <v/>
       </c>
       <c r="D23" s="13">
-        <f>'2026'!I7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
+        <f>'2026'!I10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" s="23">
       <c r="A24" s="10">
-        <f>'2026'!F8</f>
+        <f>'2026'!F11</f>
         <v/>
       </c>
       <c r="B24" s="11">
-        <f>'2026'!G8</f>
+        <f>'2026'!G11</f>
         <v/>
       </c>
       <c r="C24" s="12">
-        <f>'2026'!H8</f>
+        <f>'2026'!H11</f>
         <v/>
       </c>
       <c r="D24" s="13">
-        <f>'2026'!I8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
+        <f>'2026'!I11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" s="23">
       <c r="A25" s="10">
-        <f>'2026'!F9</f>
+        <f>'2026'!F12</f>
         <v/>
       </c>
       <c r="B25" s="11">
-        <f>'2026'!G9</f>
+        <f>'2026'!G12</f>
         <v/>
       </c>
       <c r="C25" s="12">
-        <f>'2026'!H9</f>
+        <f>'2026'!H12</f>
         <v/>
       </c>
       <c r="D25" s="13">
-        <f>'2026'!I9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
+        <f>'2026'!I12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" s="23">
       <c r="A26" s="10">
-        <f>'2026'!F10</f>
+        <f>'2026'!F13</f>
         <v/>
       </c>
       <c r="B26" s="11">
-        <f>'2026'!G10</f>
+        <f>'2026'!G13</f>
         <v/>
       </c>
       <c r="C26" s="12">
-        <f>'2026'!H10</f>
+        <f>'2026'!H13</f>
         <v/>
       </c>
       <c r="D26" s="13">
-        <f>'2026'!I10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
+        <f>'2026'!I13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" s="23">
       <c r="A27" s="10">
-        <f>'2026'!F11</f>
+        <f>'2026'!F14</f>
         <v/>
       </c>
       <c r="B27" s="11">
-        <f>'2026'!G11</f>
+        <f>'2026'!G14</f>
         <v/>
       </c>
       <c r="C27" s="12">
-        <f>'2026'!H11</f>
+        <f>'2026'!H14</f>
         <v/>
       </c>
       <c r="D27" s="13">
-        <f>'2026'!I11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
+        <f>'2026'!I14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" s="23">
       <c r="A28" s="10">
-        <f>'2026'!F12</f>
+        <f>'2026'!F15</f>
         <v/>
       </c>
       <c r="B28" s="11">
-        <f>'2026'!G12</f>
+        <f>'2026'!G15</f>
         <v/>
       </c>
       <c r="C28" s="12">
-        <f>'2026'!H12</f>
+        <f>'2026'!H15</f>
         <v/>
       </c>
       <c r="D28" s="13">
-        <f>'2026'!I12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
+        <f>'2026'!I15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" s="23">
       <c r="A29" s="10">
-        <f>'2026'!F13</f>
+        <f>'2026'!F16</f>
         <v/>
       </c>
       <c r="B29" s="11">
-        <f>'2026'!G13</f>
+        <f>'2026'!G16</f>
         <v/>
       </c>
       <c r="C29" s="12">
-        <f>'2026'!H13</f>
+        <f>'2026'!H16</f>
         <v/>
       </c>
       <c r="D29" s="13">
-        <f>'2026'!I13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="10">
-        <f>'2026'!F14</f>
-        <v/>
-      </c>
-      <c r="B30" s="11">
-        <f>'2026'!G14</f>
-        <v/>
-      </c>
-      <c r="C30" s="12">
-        <f>'2026'!H14</f>
-        <v/>
-      </c>
-      <c r="D30" s="13">
-        <f>'2026'!I14</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="10">
-        <f>'2026'!F15</f>
-        <v/>
-      </c>
-      <c r="B31" s="11">
-        <f>'2026'!G15</f>
-        <v/>
-      </c>
-      <c r="C31" s="12">
-        <f>'2026'!H15</f>
-        <v/>
-      </c>
-      <c r="D31" s="13">
-        <f>'2026'!I15</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="10">
-        <f>'2026'!F16</f>
-        <v/>
-      </c>
-      <c r="B32" s="11">
-        <f>'2026'!G16</f>
-        <v/>
-      </c>
-      <c r="C32" s="12">
-        <f>'2026'!H16</f>
-        <v/>
-      </c>
-      <c r="D32" s="13">
         <f>'2026'!I16</f>
         <v/>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="16" t="inlineStr">
+    <row r="30" s="23">
+      <c r="A30" s="16" t="inlineStr">
         <is>
           <t>Gesamt 2026</t>
         </is>
       </c>
-      <c r="B33" s="17">
+      <c r="B30" s="17">
         <f>'2026'!G17</f>
         <v/>
       </c>
-      <c r="C33" s="18">
+      <c r="C30" s="18">
         <f>'2026'!H17</f>
         <v/>
       </c>
-      <c r="D33" s="19">
+      <c r="D30" s="19">
         <f>'2026'!I17</f>
         <v/>
       </c>
     </row>
+    <row r="31" s="23"/>
+    <row r="32" s="23"/>
+    <row r="33" s="23"/>
+    <row r="34" s="23"/>
+    <row r="35" s="23"/>
+    <row r="36" s="23"/>
+    <row r="37" s="23"/>
+    <row r="38" s="23"/>
+    <row r="39" s="23"/>
   </sheetData>
-  <conditionalFormatting sqref="D3:D15">
+  <conditionalFormatting sqref="D3:D12">
     <cfRule type="expression" priority="1" dxfId="4">
       <formula>D3&lt;0</formula>
     </cfRule>
@@ -1059,12 +1019,12 @@
       <formula>D3&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D21:D33">
+  <conditionalFormatting sqref="D18:D30">
     <cfRule type="expression" priority="3" dxfId="4">
-      <formula>D21&lt;0</formula>
+      <formula>D18&lt;0</formula>
     </cfRule>
     <cfRule type="expression" priority="4" dxfId="5">
-      <formula>D21&gt;0</formula>
+      <formula>D18&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1101,42 +1061,42 @@
       <c r="A2" s="2" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1" s="23">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="24" t="inlineStr">
         <is>
           <t>Datum</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>Art</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="24" t="inlineStr">
         <is>
           <t>Was war es?</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="24" t="inlineStr">
         <is>
           <t>Betrag (€)</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="24" t="inlineStr">
         <is>
           <t>Monat 2025</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="25" t="inlineStr">
         <is>
           <t>Einnahmen (€)</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="26" t="inlineStr">
         <is>
           <t>Ausgaben (€)</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" s="24" t="inlineStr">
         <is>
           <t>Differenz (€)</t>
         </is>
@@ -4399,42 +4359,42 @@
       <c r="A2" s="2" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1" s="23">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="24" t="inlineStr">
         <is>
           <t>Datum</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>Art</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="24" t="inlineStr">
         <is>
           <t>Was war es?</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="24" t="inlineStr">
         <is>
           <t>Betrag (€)</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="24" t="inlineStr">
         <is>
           <t>Monat 2026</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="25" t="inlineStr">
         <is>
           <t>Einnahmen (€)</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="26" t="inlineStr">
         <is>
           <t>Ausgaben (€)</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" s="24" t="inlineStr">
         <is>
           <t>Differenz (€)</t>
         </is>

</xml_diff>